<commit_message>
letzte Änderung am Excel
</commit_message>
<xml_diff>
--- a/Projektwürdigkeitsanalyse_Jovo.xlsx
+++ b/Projektwürdigkeitsanalyse_Jovo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\Projektwürdigkeitsanalyse_Jovo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6111CC7B-E800-4750-9AE2-7E27DD94D212}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE8FFE7B-5361-47DA-846F-A5BA1D0CD56F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{2B98C886-53C6-4C38-874D-17CCB06E3DF5}"/>
   </bookViews>
@@ -1776,7 +1776,7 @@
     </row>
   </sheetData>
   <phoneticPr fontId="9" type="noConversion"/>
-  <dataValidations disablePrompts="1" count="12">
+  <dataValidations count="12">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J7" xr:uid="{DAA6D486-7016-45E3-BA15-5B28E5EA137E}">
       <formula1>$U$7:$W$7</formula1>
     </dataValidation>
@@ -1830,6 +1830,29 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <DocumentSetDescription xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <PA xmlns="40ef73aa-3540-4afe-b974-0f4eb1e81ef8" xsi:nil="true"/>
+    <Kontakt_Neu xmlns="40ef73aa-3540-4afe-b974-0f4eb1e81ef8">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </Kontakt_Neu>
+    <EuSGApproved xmlns="40ef73aa-3540-4afe-b974-0f4eb1e81ef8">false</EuSGApproved>
+    <TaxCatchAll xmlns="4eaf35a3-5eb2-40d3-8297-7ad4bdf1c6d5" xsi:nil="true"/>
+    <Kommentar xmlns="40ef73aa-3540-4afe-b974-0f4eb1e81ef8" xsi:nil="true"/>
+    <Bemerkung xmlns="40ef73aa-3540-4afe-b974-0f4eb1e81ef8" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="40ef73aa-3540-4afe-b974-0f4eb1e81ef8">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x0101007BED375C6DB3A84BBD73555A9A6CF129" ma:contentTypeVersion="39" ma:contentTypeDescription="Ein neues Dokument erstellen." ma:contentTypeScope="" ma:versionID="f0aef7210a4888a687ef59cdf49dff75">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="40ef73aa-3540-4afe-b974-0f4eb1e81ef8" xmlns:ns2="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns3="4eaf35a3-5eb2-40d3-8297-7ad4bdf1c6d5" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="9a3043be9839cd5df08826d9c5630a66" ns1:_="" ns2:_="" ns3:_="">
     <xsd:import namespace="40ef73aa-3540-4afe-b974-0f4eb1e81ef8"/>
@@ -2125,29 +2148,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <DocumentSetDescription xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <PA xmlns="40ef73aa-3540-4afe-b974-0f4eb1e81ef8" xsi:nil="true"/>
-    <Kontakt_Neu xmlns="40ef73aa-3540-4afe-b974-0f4eb1e81ef8">
-      <UserInfo>
-        <DisplayName/>
-        <AccountId xsi:nil="true"/>
-        <AccountType/>
-      </UserInfo>
-    </Kontakt_Neu>
-    <EuSGApproved xmlns="40ef73aa-3540-4afe-b974-0f4eb1e81ef8">false</EuSGApproved>
-    <TaxCatchAll xmlns="4eaf35a3-5eb2-40d3-8297-7ad4bdf1c6d5" xsi:nil="true"/>
-    <Kommentar xmlns="40ef73aa-3540-4afe-b974-0f4eb1e81ef8" xsi:nil="true"/>
-    <Bemerkung xmlns="40ef73aa-3540-4afe-b974-0f4eb1e81ef8" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="40ef73aa-3540-4afe-b974-0f4eb1e81ef8">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{51CF3287-B170-4086-B5C4-0449FDAF40C6}">
   <ds:schemaRefs>
@@ -2157,6 +2157,24 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4697AEC9-CCED-44FE-8C3C-145E980D06F7}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="40ef73aa-3540-4afe-b974-0f4eb1e81ef8"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="4eaf35a3-5eb2-40d3-8297-7ad4bdf1c6d5"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E0AF703C-5E45-416D-BF27-7B3A65F40DAF}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2176,24 +2194,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4697AEC9-CCED-44FE-8C3C-145E980D06F7}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="40ef73aa-3540-4afe-b974-0f4eb1e81ef8"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="4eaf35a3-5eb2-40d3-8297-7ad4bdf1c6d5"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{57d89df2-dd68-41c1-9b64-81f74f077112}" enabled="0" method="" siteId="{57d89df2-dd68-41c1-9b64-81f74f077112}" removed="1"/>

</xml_diff>